<commit_message>
The preliminary issuance register names v56 as its source
The only change in the workbook: the provenance line on the cover and in the source
note now reads CoQ_Analysis_Master_v56.xlsx instead of v55. Nothing in the register
itself moved — no Issuable state, no date, no allocation. Issuance is the owner's.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_gap_analysis/tracker/Issuance_Registers_prelim.xlsx
+++ b/deliverables/qc_gap_analysis/tracker/Issuance_Registers_prelim.xlsx
@@ -55002,7 +55002,7 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>iCoA and CoQ Issuance Registers — preliminary — built with CoQ Analysis Master v55 on 21.09.2026</t>
+          <t>iCoA and CoQ Issuance Registers — preliminary — built with CoQ Analysis Master v56 on 21.09.2026</t>
         </is>
       </c>
     </row>
@@ -55023,7 +55023,7 @@
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Source: CoQ_Analysis_Master_v55.xlsx, sheets iCoA Register and Batch Dates; dates from the Head of QC's list of 04.09.2026; the issuance plan of 31.08.2026 for the plan references.</t>
+          <t>Source: CoQ_Analysis_Master_v56.xlsx, sheets iCoA Register and Batch Dates; dates from the Head of QC's list of 04.09.2026; the issuance plan of 31.08.2026 for the plan references.</t>
         </is>
       </c>
     </row>

</xml_diff>